<commit_message>
🤖 ZenPro v3.2 · 24 Mar 2026 19:51 IST · IN:1bull/0sell · US:1bull
</commit_message>
<xml_diff>
--- a/ZenPro_v3_Signals.xlsx
+++ b/ZenPro_v3_Signals.xlsx
@@ -909,7 +909,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="23" t="inlineStr">
         <is>
-          <t>⚡ ZENPRO v3.2 · RATIOS · Gold=4388 DXY=99.40 · 24 Mar 2026</t>
+          <t>⚡ ZENPRO v3.2 · RATIOS · Gold=4401 DXY=99.33 · 24 Mar 2026</t>
         </is>
       </c>
     </row>
@@ -947,10 +947,10 @@
         </is>
       </c>
       <c r="B3" s="29" t="n">
-        <v>5.2217</v>
+        <v>5.2065</v>
       </c>
       <c r="C3" s="30" t="n">
-        <v>230.51</v>
+        <v>230.66</v>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
@@ -970,10 +970,10 @@
         </is>
       </c>
       <c r="B4" s="29" t="n">
-        <v>11.9888</v>
+        <v>11.9539</v>
       </c>
       <c r="C4" s="30" t="n">
-        <v>529.24</v>
+        <v>529.59</v>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
@@ -993,10 +993,10 @@
         </is>
       </c>
       <c r="B5" s="29" t="n">
-        <v>6.757</v>
+        <v>6.7373</v>
       </c>
       <c r="C5" s="30" t="n">
-        <v>298.28</v>
+        <v>298.48</v>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="B6" s="29" t="n">
-        <v>5.587</v>
+        <v>5.5708</v>
       </c>
       <c r="C6" s="30" t="n">
-        <v>246.63</v>
+        <v>246.8</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
@@ -1039,10 +1039,10 @@
         </is>
       </c>
       <c r="B7" s="29" t="n">
-        <v>5.0684</v>
+        <v>5.0537</v>
       </c>
       <c r="C7" s="30" t="n">
-        <v>223.74</v>
+        <v>223.89</v>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
@@ -1062,10 +1062,10 @@
         </is>
       </c>
       <c r="B8" s="29" t="n">
-        <v>10.5764</v>
+        <v>10.5457</v>
       </c>
       <c r="C8" s="30" t="n">
-        <v>466.89</v>
+        <v>467.2</v>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
@@ -1085,10 +1085,10 @@
         </is>
       </c>
       <c r="B9" s="29" t="n">
-        <v>2.5204</v>
+        <v>2.513</v>
       </c>
       <c r="C9" s="30" t="n">
-        <v>111.26</v>
+        <v>111.34</v>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="B10" s="29" t="n">
-        <v>0.1536</v>
+        <v>0.1531</v>
       </c>
       <c r="C10" s="30" t="n">
         <v>6.78</v>
@@ -1131,10 +1131,10 @@
         </is>
       </c>
       <c r="B11" s="29" t="n">
-        <v>7.9953</v>
+        <v>7.972</v>
       </c>
       <c r="C11" s="30" t="n">
-        <v>352.95</v>
+        <v>353.18</v>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
@@ -1154,10 +1154,10 @@
         </is>
       </c>
       <c r="B12" s="29" t="n">
-        <v>0.2955</v>
+        <v>0.2946</v>
       </c>
       <c r="C12" s="30" t="n">
-        <v>13.04</v>
+        <v>13.05</v>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
@@ -1177,10 +1177,10 @@
         </is>
       </c>
       <c r="B13" s="29" t="n">
-        <v>1.9905</v>
+        <v>1.9847</v>
       </c>
       <c r="C13" s="30" t="n">
-        <v>87.87</v>
+        <v>87.93000000000001</v>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
@@ -1200,10 +1200,10 @@
         </is>
       </c>
       <c r="B14" s="29" t="n">
-        <v>1.9047</v>
+        <v>1.8991</v>
       </c>
       <c r="C14" s="30" t="n">
-        <v>84.08</v>
+        <v>84.14</v>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
@@ -1223,10 +1223,10 @@
         </is>
       </c>
       <c r="B15" s="29" t="n">
-        <v>3.5123</v>
+        <v>3.5021</v>
       </c>
       <c r="C15" s="30" t="n">
-        <v>155.05</v>
+        <v>155.15</v>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
@@ -1345,7 +1345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1435,13 +1435,13 @@
         </is>
       </c>
       <c r="E3" s="6" t="n">
-        <v>116.46</v>
+        <v>115.71</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>51.7</v>
+        <v>49.1</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
@@ -1449,52 +1449,52 @@
         </is>
       </c>
       <c r="I3" s="5" t="n">
-        <v>0.68</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>MRK</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>Daily</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>🟢 Sq20/50</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>🐂BULL</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>116.46</v>
-      </c>
-      <c r="F4" s="7" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="G4" s="8" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>🟣 MACD↓</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>🐻BEAR</t>
+        </is>
+      </c>
+      <c r="E4" s="19" t="n">
+        <v>296.41</v>
+      </c>
+      <c r="F4" s="20" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="G4" s="21" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>ABOVE</t>
         </is>
       </c>
-      <c r="I4" s="5" t="n">
-        <v>0.68</v>
+      <c r="I4" s="18" t="n">
+        <v>-1.87</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B5" s="16" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="C5" s="17" t="inlineStr">
         <is>
-          <t>🟣 MACD↓</t>
+          <t>🟠 RSI/SMA↓</t>
         </is>
       </c>
       <c r="D5" s="18" t="inlineStr">
@@ -1513,27 +1513,27 @@
         </is>
       </c>
       <c r="E5" s="19" t="n">
-        <v>296.47</v>
+        <v>207.85</v>
       </c>
       <c r="F5" s="20" t="n">
-        <v>37.9</v>
+        <v>44.5</v>
       </c>
       <c r="G5" s="21" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="H5" s="22" t="inlineStr">
-        <is>
-          <t>ABOVE</t>
+        <v>0.12</v>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>BELOW</t>
         </is>
       </c>
       <c r="I5" s="18" t="n">
-        <v>-1.85</v>
+        <v>-1.09</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
-          <t>🟠 RSI/SMA↓</t>
+          <t>🔴 MACD 0↓</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
@@ -1552,60 +1552,21 @@
         </is>
       </c>
       <c r="E6" s="19" t="n">
-        <v>207.55</v>
+        <v>234.46</v>
       </c>
       <c r="F6" s="20" t="n">
-        <v>44.2</v>
+        <v>40.8</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="H6" s="18" t="inlineStr">
-        <is>
-          <t>BELOW</t>
+        <v>0.1</v>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t>ABOVE</t>
         </is>
       </c>
       <c r="I6" s="18" t="n">
-        <v>-1.23</v>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>JNJ</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>Daily</t>
-        </is>
-      </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>🔴 MACD 0↓</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>🐻BEAR</t>
-        </is>
-      </c>
-      <c r="E7" s="19" t="n">
-        <v>235.32</v>
-      </c>
-      <c r="F7" s="20" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="G7" s="21" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="H7" s="22" t="inlineStr">
-        <is>
-          <t>ABOVE</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="n">
-        <v>-0.04</v>
+        <v>-0.41</v>
       </c>
     </row>
   </sheetData>
@@ -1714,7 +1675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2325,76 +2286,76 @@
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>BANDHANBNK</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="n">
+        <v>149.99</v>
+      </c>
+      <c r="C26" s="30" t="n">
+        <v>8123440</v>
+      </c>
+      <c r="D26" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="35" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F26" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+      <c r="G26" s="34" t="n">
+        <v>1.11</v>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>FEDERALBNK</t>
         </is>
       </c>
-      <c r="B26" s="36" t="n">
+      <c r="B27" s="36" t="n">
         <v>262.5</v>
       </c>
-      <c r="C26" s="14" t="n">
+      <c r="C27" s="14" t="n">
         <v>6879978</v>
       </c>
-      <c r="D26" s="4" t="n">
+      <c r="D27" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="37" t="n">
+      <c r="E27" s="37" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>ABOVE</t>
         </is>
       </c>
-      <c r="G26" s="5" t="n">
+      <c r="G27" s="5" t="n">
         <v>3.2</v>
-      </c>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="28" t="inlineStr">
-        <is>
-          <t>INDHOTEL</t>
-        </is>
-      </c>
-      <c r="B27" s="29" t="n">
-        <v>604.05</v>
-      </c>
-      <c r="C27" s="30" t="n">
-        <v>2989995</v>
-      </c>
-      <c r="D27" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="35" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="F27" s="33" t="inlineStr">
-        <is>
-          <t>BELOW</t>
-        </is>
-      </c>
-      <c r="G27" s="34" t="n">
-        <v>3.71</v>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="28" t="inlineStr">
         <is>
-          <t>CONCOR</t>
+          <t>INDHOTEL</t>
         </is>
       </c>
       <c r="B28" s="29" t="n">
-        <v>433.1</v>
+        <v>604.05</v>
       </c>
       <c r="C28" s="30" t="n">
-        <v>2423789</v>
+        <v>2989995</v>
       </c>
       <c r="D28" s="31" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="35" t="n">
-        <v>1.65</v>
+        <v>1.15</v>
       </c>
       <c r="F28" s="33" t="inlineStr">
         <is>
@@ -2402,26 +2363,26 @@
         </is>
       </c>
       <c r="G28" s="34" t="n">
-        <v>2.21</v>
+        <v>3.71</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="28" t="inlineStr">
         <is>
-          <t>AVANTEL</t>
+          <t>CONCOR</t>
         </is>
       </c>
       <c r="B29" s="29" t="n">
-        <v>121.03</v>
+        <v>433.1</v>
       </c>
       <c r="C29" s="30" t="n">
-        <v>1810186</v>
+        <v>2423789</v>
       </c>
       <c r="D29" s="31" t="n">
         <v>0</v>
       </c>
       <c r="E29" s="35" t="n">
-        <v>1.51</v>
+        <v>1.65</v>
       </c>
       <c r="F29" s="33" t="inlineStr">
         <is>
@@ -2429,26 +2390,26 @@
         </is>
       </c>
       <c r="G29" s="34" t="n">
-        <v>2.32</v>
+        <v>2.21</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="28" t="inlineStr">
         <is>
-          <t>MFSL</t>
+          <t>AVANTEL</t>
         </is>
       </c>
       <c r="B30" s="29" t="n">
-        <v>1583.5</v>
+        <v>121.03</v>
       </c>
       <c r="C30" s="30" t="n">
-        <v>1556964</v>
+        <v>1810186</v>
       </c>
       <c r="D30" s="31" t="n">
         <v>0</v>
       </c>
       <c r="E30" s="35" t="n">
-        <v>1.74</v>
+        <v>1.51</v>
       </c>
       <c r="F30" s="33" t="inlineStr">
         <is>
@@ -2456,26 +2417,26 @@
         </is>
       </c>
       <c r="G30" s="34" t="n">
-        <v>1.02</v>
+        <v>2.32</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="28" t="inlineStr">
         <is>
-          <t>SRF</t>
+          <t>MFSL</t>
         </is>
       </c>
       <c r="B31" s="29" t="n">
-        <v>2471.6</v>
+        <v>1583.5</v>
       </c>
       <c r="C31" s="30" t="n">
-        <v>1285209</v>
+        <v>1556964</v>
       </c>
       <c r="D31" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="E31" s="32" t="n">
-        <v>2.43</v>
+      <c r="E31" s="35" t="n">
+        <v>1.74</v>
       </c>
       <c r="F31" s="33" t="inlineStr">
         <is>
@@ -2483,33 +2444,60 @@
         </is>
       </c>
       <c r="G31" s="34" t="n">
-        <v>3.35</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="28" t="inlineStr">
         <is>
-          <t>LXCHEM</t>
+          <t>SRF</t>
         </is>
       </c>
       <c r="B32" s="29" t="n">
-        <v>118</v>
+        <v>2471.6</v>
       </c>
       <c r="C32" s="30" t="n">
-        <v>1161733</v>
+        <v>1285209</v>
       </c>
       <c r="D32" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="E32" s="35" t="n">
+      <c r="E32" s="32" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="F32" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+      <c r="G32" s="34" t="n">
+        <v>3.35</v>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="28" t="inlineStr">
+        <is>
+          <t>LXCHEM</t>
+        </is>
+      </c>
+      <c r="B33" s="29" t="n">
+        <v>118</v>
+      </c>
+      <c r="C33" s="30" t="n">
+        <v>1161733</v>
+      </c>
+      <c r="D33" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="35" t="n">
         <v>1.45</v>
       </c>
-      <c r="F32" s="33" t="inlineStr">
-        <is>
-          <t>BELOW</t>
-        </is>
-      </c>
-      <c r="G32" s="34" t="n">
+      <c r="F33" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+      <c r="G33" s="34" t="n">
         <v>4.52</v>
       </c>
     </row>
@@ -2530,7 +2518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2604,68 +2592,68 @@
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>NAVINFLUOR</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="n">
+        <v>6184.5</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>6965</v>
+      </c>
+      <c r="D8" s="42" t="n">
+        <v>6649.5</v>
+      </c>
+      <c r="E8" s="37" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>ABOVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
           <t>THANGAMAYL</t>
         </is>
       </c>
-      <c r="B8" s="36" t="n">
+      <c r="B9" s="36" t="n">
         <v>3309.4</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C9" s="5" t="n">
         <v>4149</v>
       </c>
-      <c r="D8" s="42" t="n">
+      <c r="D9" s="42" t="n">
         <v>3959.2</v>
       </c>
-      <c r="E8" s="37" t="n">
+      <c r="E9" s="37" t="n">
         <v>41.7</v>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>ABOVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="28" t="inlineStr">
-        <is>
-          <t>SRF</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="n">
-        <v>2471.6</v>
-      </c>
-      <c r="C9" s="34" t="n">
-        <v>3325</v>
-      </c>
-      <c r="D9" s="32" t="n">
-        <v>3276.15</v>
-      </c>
-      <c r="E9" s="35" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="F9" s="33" t="inlineStr">
-        <is>
-          <t>BELOW</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="28" t="inlineStr">
         <is>
-          <t>MFSL</t>
+          <t>SRF</t>
         </is>
       </c>
       <c r="B10" s="29" t="n">
-        <v>1583.5</v>
+        <v>2471.6</v>
       </c>
       <c r="C10" s="34" t="n">
-        <v>1892.5</v>
+        <v>3325</v>
       </c>
       <c r="D10" s="32" t="n">
-        <v>1870</v>
+        <v>3276.15</v>
       </c>
       <c r="E10" s="35" t="n">
-        <v>33.4</v>
+        <v>42.3</v>
       </c>
       <c r="F10" s="33" t="inlineStr">
         <is>
@@ -2674,72 +2662,168 @@
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="28" t="inlineStr">
-        <is>
-          <t>RELIANCE</t>
-        </is>
-      </c>
-      <c r="B11" s="29" t="n">
-        <v>1411.8</v>
-      </c>
-      <c r="C11" s="34" t="n">
-        <v>1611.8</v>
-      </c>
-      <c r="D11" s="32" t="n">
-        <v>1592.3</v>
-      </c>
-      <c r="E11" s="35" t="n">
-        <v>50.9</v>
-      </c>
-      <c r="F11" s="33" t="inlineStr">
-        <is>
-          <t>BELOW</t>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>GLENMARK</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="n">
+        <v>2095.7</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>2297.9</v>
+      </c>
+      <c r="D11" s="42" t="n">
+        <v>2272.7</v>
+      </c>
+      <c r="E11" s="37" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>ABOVE</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="28" t="inlineStr">
         <is>
+          <t>MFSL</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="n">
+        <v>1583.5</v>
+      </c>
+      <c r="C12" s="34" t="n">
+        <v>1892.5</v>
+      </c>
+      <c r="D12" s="32" t="n">
+        <v>1870</v>
+      </c>
+      <c r="E12" s="35" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="F12" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="n">
+        <v>1411.8</v>
+      </c>
+      <c r="C13" s="34" t="n">
+        <v>1611.8</v>
+      </c>
+      <c r="D13" s="32" t="n">
+        <v>1592.3</v>
+      </c>
+      <c r="E13" s="35" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="F13" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>WELCORP</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="n">
+        <v>802.2</v>
+      </c>
+      <c r="C14" s="34" t="n">
+        <v>994</v>
+      </c>
+      <c r="D14" s="32" t="n">
+        <v>965.75</v>
+      </c>
+      <c r="E14" s="35" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="F14" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
           <t>KIMS</t>
         </is>
       </c>
-      <c r="B12" s="29" t="n">
+      <c r="B15" s="29" t="n">
         <v>631.05</v>
       </c>
-      <c r="C12" s="34" t="n">
+      <c r="C15" s="34" t="n">
         <v>798.4</v>
       </c>
-      <c r="D12" s="32" t="n">
+      <c r="D15" s="32" t="n">
         <v>789.35</v>
       </c>
-      <c r="E12" s="35" t="n">
+      <c r="E15" s="35" t="n">
         <v>39.1</v>
       </c>
-      <c r="F12" s="33" t="inlineStr">
-        <is>
-          <t>BELOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="F15" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>GRAPHITE</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="n">
+        <v>570.85</v>
+      </c>
+      <c r="C16" s="34" t="n">
+        <v>747</v>
+      </c>
+      <c r="D16" s="32" t="n">
+        <v>730.15</v>
+      </c>
+      <c r="E16" s="35" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="F16" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>FEDERALBNK</t>
         </is>
       </c>
-      <c r="B13" s="36" t="n">
+      <c r="B17" s="36" t="n">
         <v>262.5</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C17" s="5" t="n">
         <v>302</v>
       </c>
-      <c r="D13" s="42" t="n">
+      <c r="D17" s="42" t="n">
         <v>299.85</v>
       </c>
-      <c r="E13" s="37" t="n">
+      <c r="E17" s="37" t="n">
         <v>40.4</v>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>ABOVE</t>
         </is>
@@ -2763,7 +2847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2845,98 +2929,98 @@
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="31" t="n">
+      <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>NAVINFLUOR</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>92.40000000000001</v>
+      </c>
+      <c r="D5" s="36" t="n">
+        <v>6184.5</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>ABOVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
         <is>
           <t>MFSL</t>
         </is>
       </c>
-      <c r="C5" s="34" t="n">
+      <c r="C6" s="34" t="n">
         <v>87.5</v>
       </c>
-      <c r="D5" s="29" t="n">
+      <c r="D6" s="29" t="n">
         <v>1583.5</v>
       </c>
-      <c r="E5" s="34" t="n">
+      <c r="E6" s="34" t="n">
         <v>1.02</v>
       </c>
-      <c r="F5" s="33" t="inlineStr">
-        <is>
-          <t>BELOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="F6" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>FEDERALBNK</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C7" s="5" t="n">
         <v>86</v>
       </c>
-      <c r="D6" s="36" t="n">
+      <c r="D7" s="36" t="n">
         <v>262.5</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E7" s="5" t="n">
         <v>3.2</v>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>ABOVE</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="31" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="28" t="inlineStr">
-        <is>
-          <t>SURYODAY</t>
-        </is>
-      </c>
-      <c r="C7" s="34" t="n">
-        <v>70</v>
-      </c>
-      <c r="D7" s="29" t="n">
-        <v>125.53</v>
-      </c>
-      <c r="E7" s="34" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="F7" s="33" t="inlineStr">
-        <is>
-          <t>BELOW</t>
-        </is>
-      </c>
-    </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="31" t="n">
+      <c r="A8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="28" t="inlineStr">
-        <is>
-          <t>RELIANCE</t>
-        </is>
-      </c>
-      <c r="C8" s="29" t="n">
-        <v>63.4</v>
-      </c>
-      <c r="D8" s="29" t="n">
-        <v>1411.8</v>
-      </c>
-      <c r="E8" s="34" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="F8" s="33" t="inlineStr">
-        <is>
-          <t>BELOW</t>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>GLENMARK</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="D8" s="36" t="n">
+        <v>2095.7</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>ABOVE</t>
         </is>
       </c>
     </row>
@@ -2946,17 +3030,17 @@
       </c>
       <c r="B9" s="28" t="inlineStr">
         <is>
-          <t>RATEGAIN</t>
-        </is>
-      </c>
-      <c r="C9" s="29" t="n">
-        <v>61.2</v>
+          <t>GRAPHITE</t>
+        </is>
+      </c>
+      <c r="C9" s="34" t="n">
+        <v>73.5</v>
       </c>
       <c r="D9" s="29" t="n">
-        <v>480.85</v>
+        <v>570.85</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>3.02</v>
+        <v>1.27</v>
       </c>
       <c r="F9" s="33" t="inlineStr">
         <is>
@@ -2970,17 +3054,17 @@
       </c>
       <c r="B10" s="28" t="inlineStr">
         <is>
-          <t>METROPOLIS</t>
-        </is>
-      </c>
-      <c r="C10" s="29" t="n">
-        <v>60</v>
+          <t>SURYODAY</t>
+        </is>
+      </c>
+      <c r="C10" s="34" t="n">
+        <v>70</v>
       </c>
       <c r="D10" s="29" t="n">
-        <v>443</v>
-      </c>
-      <c r="E10" s="33" t="n">
-        <v>-1.6</v>
+        <v>125.53</v>
+      </c>
+      <c r="E10" s="34" t="n">
+        <v>0.13</v>
       </c>
       <c r="F10" s="33" t="inlineStr">
         <is>
@@ -2994,17 +3078,17 @@
       </c>
       <c r="B11" s="28" t="inlineStr">
         <is>
-          <t>AVANTEL</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="C11" s="29" t="n">
-        <v>58.2</v>
+        <v>63.4</v>
       </c>
       <c r="D11" s="29" t="n">
-        <v>121.03</v>
+        <v>1411.8</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>2.32</v>
+        <v>0.28</v>
       </c>
       <c r="F11" s="33" t="inlineStr">
         <is>
@@ -3018,17 +3102,17 @@
       </c>
       <c r="B12" s="28" t="inlineStr">
         <is>
-          <t>KIMS</t>
+          <t>RATEGAIN</t>
         </is>
       </c>
       <c r="C12" s="29" t="n">
-        <v>58</v>
+        <v>61.2</v>
       </c>
       <c r="D12" s="29" t="n">
-        <v>631.05</v>
+        <v>480.85</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>0.09</v>
+        <v>3.02</v>
       </c>
       <c r="F12" s="33" t="inlineStr">
         <is>
@@ -3037,26 +3121,26 @@
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>AARTIIND</t>
-        </is>
-      </c>
-      <c r="C13" s="36" t="n">
-        <v>56.6</v>
-      </c>
-      <c r="D13" s="36" t="n">
-        <v>418.7</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>3.34</v>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>ABOVE</t>
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>METROPOLIS</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="n">
+        <v>60</v>
+      </c>
+      <c r="D13" s="29" t="n">
+        <v>443</v>
+      </c>
+      <c r="E13" s="33" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="F13" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
         </is>
       </c>
     </row>
@@ -3066,17 +3150,17 @@
       </c>
       <c r="B14" s="28" t="inlineStr">
         <is>
-          <t>DMART</t>
+          <t>AVANTEL</t>
         </is>
       </c>
       <c r="C14" s="29" t="n">
-        <v>50.7</v>
+        <v>58.2</v>
       </c>
       <c r="D14" s="29" t="n">
-        <v>3756.5</v>
+        <v>121.03</v>
       </c>
       <c r="E14" s="34" t="n">
-        <v>2.76</v>
+        <v>2.32</v>
       </c>
       <c r="F14" s="33" t="inlineStr">
         <is>
@@ -3090,17 +3174,17 @@
       </c>
       <c r="B15" s="28" t="inlineStr">
         <is>
-          <t>TORNTPOWER</t>
-        </is>
-      </c>
-      <c r="C15" s="33" t="n">
-        <v>49.5</v>
+          <t>BANDHANBNK</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="n">
+        <v>58.2</v>
       </c>
       <c r="D15" s="29" t="n">
-        <v>1366.3</v>
+        <v>149.99</v>
       </c>
       <c r="E15" s="34" t="n">
-        <v>0.26</v>
+        <v>1.11</v>
       </c>
       <c r="F15" s="33" t="inlineStr">
         <is>
@@ -3114,17 +3198,17 @@
       </c>
       <c r="B16" s="28" t="inlineStr">
         <is>
-          <t>KOLTEPATIL</t>
-        </is>
-      </c>
-      <c r="C16" s="33" t="n">
-        <v>47.8</v>
+          <t>KIMS</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="n">
+        <v>58</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>322.25</v>
-      </c>
-      <c r="E16" s="33" t="n">
-        <v>-0.26</v>
+        <v>631.05</v>
+      </c>
+      <c r="E16" s="34" t="n">
+        <v>0.09</v>
       </c>
       <c r="F16" s="33" t="inlineStr">
         <is>
@@ -3133,26 +3217,26 @@
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="31" t="n">
+      <c r="A17" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="28" t="inlineStr">
-        <is>
-          <t>MANKIND</t>
-        </is>
-      </c>
-      <c r="C17" s="33" t="n">
-        <v>46.1</v>
-      </c>
-      <c r="D17" s="29" t="n">
-        <v>1987.8</v>
-      </c>
-      <c r="E17" s="34" t="n">
-        <v>3.13</v>
-      </c>
-      <c r="F17" s="33" t="inlineStr">
-        <is>
-          <t>BELOW</t>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>AARTIIND</t>
+        </is>
+      </c>
+      <c r="C17" s="36" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="D17" s="36" t="n">
+        <v>418.7</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>ABOVE</t>
         </is>
       </c>
     </row>
@@ -3162,17 +3246,17 @@
       </c>
       <c r="B18" s="28" t="inlineStr">
         <is>
-          <t>SRF</t>
-        </is>
-      </c>
-      <c r="C18" s="33" t="n">
-        <v>38.5</v>
+          <t>WELCORP</t>
+        </is>
+      </c>
+      <c r="C18" s="29" t="n">
+        <v>52.2</v>
       </c>
       <c r="D18" s="29" t="n">
-        <v>2471.6</v>
+        <v>802.2</v>
       </c>
       <c r="E18" s="34" t="n">
-        <v>3.35</v>
+        <v>4.05</v>
       </c>
       <c r="F18" s="33" t="inlineStr">
         <is>
@@ -3186,17 +3270,17 @@
       </c>
       <c r="B19" s="28" t="inlineStr">
         <is>
-          <t>TANLA</t>
-        </is>
-      </c>
-      <c r="C19" s="33" t="n">
-        <v>37.1</v>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="n">
+        <v>50.7</v>
       </c>
       <c r="D19" s="29" t="n">
-        <v>410.95</v>
+        <v>3756.5</v>
       </c>
       <c r="E19" s="34" t="n">
-        <v>2.74</v>
+        <v>2.76</v>
       </c>
       <c r="F19" s="33" t="inlineStr">
         <is>
@@ -3210,17 +3294,17 @@
       </c>
       <c r="B20" s="28" t="inlineStr">
         <is>
-          <t>CONCOR</t>
+          <t>TORNTPOWER</t>
         </is>
       </c>
       <c r="C20" s="33" t="n">
-        <v>36.9</v>
+        <v>49.5</v>
       </c>
       <c r="D20" s="29" t="n">
-        <v>433.1</v>
+        <v>1366.3</v>
       </c>
       <c r="E20" s="34" t="n">
-        <v>2.21</v>
+        <v>0.26</v>
       </c>
       <c r="F20" s="33" t="inlineStr">
         <is>
@@ -3234,17 +3318,17 @@
       </c>
       <c r="B21" s="28" t="inlineStr">
         <is>
-          <t>SAFARI</t>
+          <t>KOLTEPATIL</t>
         </is>
       </c>
       <c r="C21" s="33" t="n">
-        <v>32.6</v>
+        <v>47.8</v>
       </c>
       <c r="D21" s="29" t="n">
-        <v>1479.3</v>
+        <v>322.25</v>
       </c>
       <c r="E21" s="33" t="n">
-        <v>-0.24</v>
+        <v>-0.26</v>
       </c>
       <c r="F21" s="33" t="inlineStr">
         <is>
@@ -3258,17 +3342,17 @@
       </c>
       <c r="B22" s="28" t="inlineStr">
         <is>
-          <t>INDHOTEL</t>
+          <t>MANKIND</t>
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>32.3</v>
+        <v>46.1</v>
       </c>
       <c r="D22" s="29" t="n">
-        <v>604.05</v>
+        <v>1987.8</v>
       </c>
       <c r="E22" s="34" t="n">
-        <v>3.71</v>
+        <v>3.13</v>
       </c>
       <c r="F22" s="33" t="inlineStr">
         <is>
@@ -3282,17 +3366,17 @@
       </c>
       <c r="B23" s="28" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>SRF</t>
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>28.9</v>
+        <v>38.5</v>
       </c>
       <c r="D23" s="29" t="n">
-        <v>1334.3</v>
+        <v>2471.6</v>
       </c>
       <c r="E23" s="34" t="n">
-        <v>0.34</v>
+        <v>3.35</v>
       </c>
       <c r="F23" s="33" t="inlineStr">
         <is>
@@ -3306,17 +3390,17 @@
       </c>
       <c r="B24" s="28" t="inlineStr">
         <is>
-          <t>LXCHEM</t>
+          <t>TANLA</t>
         </is>
       </c>
       <c r="C24" s="33" t="n">
-        <v>25.1</v>
+        <v>37.1</v>
       </c>
       <c r="D24" s="29" t="n">
-        <v>118</v>
+        <v>410.95</v>
       </c>
       <c r="E24" s="34" t="n">
-        <v>4.52</v>
+        <v>2.74</v>
       </c>
       <c r="F24" s="33" t="inlineStr">
         <is>
@@ -3330,17 +3414,17 @@
       </c>
       <c r="B25" s="28" t="inlineStr">
         <is>
-          <t>BAJAJHFL</t>
+          <t>CONCOR</t>
         </is>
       </c>
       <c r="C25" s="33" t="n">
-        <v>24.3</v>
+        <v>36.9</v>
       </c>
       <c r="D25" s="29" t="n">
-        <v>78.75</v>
+        <v>433.1</v>
       </c>
       <c r="E25" s="34" t="n">
-        <v>0.31</v>
+        <v>2.21</v>
       </c>
       <c r="F25" s="33" t="inlineStr">
         <is>
@@ -3354,17 +3438,17 @@
       </c>
       <c r="B26" s="28" t="inlineStr">
         <is>
-          <t>PDSL</t>
+          <t>SAFARI</t>
         </is>
       </c>
       <c r="C26" s="33" t="n">
-        <v>22.1</v>
+        <v>32.6</v>
       </c>
       <c r="D26" s="29" t="n">
-        <v>274.05</v>
-      </c>
-      <c r="E26" s="34" t="n">
-        <v>7.96</v>
+        <v>1479.3</v>
+      </c>
+      <c r="E26" s="33" t="n">
+        <v>-0.24</v>
       </c>
       <c r="F26" s="33" t="inlineStr">
         <is>
@@ -3378,19 +3462,139 @@
       </c>
       <c r="B27" s="28" t="inlineStr">
         <is>
+          <t>INDHOTEL</t>
+        </is>
+      </c>
+      <c r="C27" s="33" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="D27" s="29" t="n">
+        <v>604.05</v>
+      </c>
+      <c r="E27" s="34" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="F27" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="31" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t>ACC</t>
+        </is>
+      </c>
+      <c r="C28" s="33" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="D28" s="29" t="n">
+        <v>1334.3</v>
+      </c>
+      <c r="E28" s="34" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="F28" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="31" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="28" t="inlineStr">
+        <is>
+          <t>LXCHEM</t>
+        </is>
+      </c>
+      <c r="C29" s="33" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="D29" s="29" t="n">
+        <v>118</v>
+      </c>
+      <c r="E29" s="34" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="F29" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="31" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="28" t="inlineStr">
+        <is>
+          <t>BAJAJHFL</t>
+        </is>
+      </c>
+      <c r="C30" s="33" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="D30" s="29" t="n">
+        <v>78.75</v>
+      </c>
+      <c r="E30" s="34" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F30" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="31" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="28" t="inlineStr">
+        <is>
+          <t>PDSL</t>
+        </is>
+      </c>
+      <c r="C31" s="33" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="D31" s="29" t="n">
+        <v>274.05</v>
+      </c>
+      <c r="E31" s="34" t="n">
+        <v>7.96</v>
+      </c>
+      <c r="F31" s="33" t="inlineStr">
+        <is>
+          <t>BELOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="28" t="inlineStr">
+        <is>
           <t>LODHA</t>
         </is>
       </c>
-      <c r="C27" s="33" t="n">
+      <c r="C32" s="33" t="n">
         <v>22</v>
       </c>
-      <c r="D27" s="29" t="n">
+      <c r="D32" s="29" t="n">
         <v>726.4</v>
       </c>
-      <c r="E27" s="33" t="n">
+      <c r="E32" s="33" t="n">
         <v>-0.21</v>
       </c>
-      <c r="F27" s="33" t="inlineStr">
+      <c r="F32" s="33" t="inlineStr">
         <is>
           <t>BELOW</t>
         </is>
@@ -3412,7 +3616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3505,242 +3709,377 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="28" t="inlineStr">
         <is>
-          <t>Mirae Asset Large &amp; Midcap Fund - Direct Plan - Growth</t>
+          <t>quant Small Cap Fund - Growth Option - Direct Plan</t>
         </is>
       </c>
       <c r="B5" s="45" t="n">
-        <v>160.17</v>
+        <v>248.64</v>
       </c>
       <c r="C5" s="46" t="n">
-        <v>3.98</v>
+        <v>-1.88</v>
       </c>
       <c r="D5" s="46" t="n">
-        <v>16.99</v>
+        <v>19.88</v>
       </c>
       <c r="E5" s="46" t="n">
-        <v>14.24</v>
+        <v>24.55</v>
       </c>
       <c r="F5" s="47" t="n">
-        <v>18.01</v>
+        <v>18.57</v>
       </c>
       <c r="G5" s="48" t="inlineStr">
         <is>
-          <t>Equity Scheme - Large &amp; Mid Cap Fund</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="49" t="inlineStr">
-        <is>
-          <t>— ETFs &amp; BeES —</t>
+          <t>Equity Scheme - Small Cap Fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>Franklin India Mid Cap Fund - Direct - Growth</t>
+        </is>
+      </c>
+      <c r="B6" s="45" t="n">
+        <v>2807</v>
+      </c>
+      <c r="C6" s="46" t="n">
+        <v>-1.15</v>
+      </c>
+      <c r="D6" s="46" t="n">
+        <v>20.77</v>
+      </c>
+      <c r="E6" s="46" t="n">
+        <v>16.36</v>
+      </c>
+      <c r="F6" s="47" t="n">
+        <v>15.51</v>
+      </c>
+      <c r="G6" s="48" t="inlineStr">
+        <is>
+          <t>Equity Scheme - Mid Cap Fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>CANARA ROBECO EQUITY HYBRID FUND - DIRECT PLAN - GROWTH OPTION</t>
+        </is>
+      </c>
+      <c r="B7" s="45" t="n">
+        <v>390.65</v>
+      </c>
+      <c r="C7" s="46" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="D7" s="46" t="n">
+        <v>13.93</v>
+      </c>
+      <c r="E7" s="46" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="F7" s="45" t="n">
+        <v>13.64</v>
+      </c>
+      <c r="G7" s="48" t="inlineStr">
+        <is>
+          <t>Hybrid Scheme - Aggressive Hybrid Fund</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="28" t="inlineStr">
         <is>
-          <t>Nifty BeES</t>
-        </is>
-      </c>
-      <c r="B8" s="29" t="n">
-        <v>259.83</v>
-      </c>
-      <c r="C8" s="35" t="n">
-        <v>3.03</v>
-      </c>
-      <c r="D8" s="35" t="n">
-        <v>36.97</v>
-      </c>
-      <c r="E8" s="35" t="n">
-        <v>68.87</v>
-      </c>
-      <c r="F8" s="35" t="inlineStr"/>
+          <t>Axis Large Cap Fund - Direct Plan - Growth</t>
+        </is>
+      </c>
+      <c r="B8" s="45" t="n">
+        <v>64.36</v>
+      </c>
+      <c r="C8" s="46" t="n">
+        <v>-2.59</v>
+      </c>
+      <c r="D8" s="46" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="E8" s="46" t="n">
+        <v>9.08</v>
+      </c>
+      <c r="F8" s="45" t="n">
+        <v>13.05</v>
+      </c>
+      <c r="G8" s="48" t="inlineStr">
+        <is>
+          <t>Equity Scheme - Large Cap Fund</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="28" t="inlineStr">
         <is>
-          <t>Bank BeES</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="n">
-        <v>543.04</v>
-      </c>
-      <c r="C9" s="35" t="n">
-        <v>9.51</v>
-      </c>
-      <c r="D9" s="35" t="n">
-        <v>33.08</v>
-      </c>
-      <c r="E9" s="35" t="n">
-        <v>63.06</v>
-      </c>
-      <c r="F9" s="35" t="inlineStr"/>
+          <t>Axis ELSS Tax Saver Fund - Direct Plan - Growth Option</t>
+        </is>
+      </c>
+      <c r="B9" s="45" t="n">
+        <v>99.61</v>
+      </c>
+      <c r="C9" s="46" t="n">
+        <v>-2.83</v>
+      </c>
+      <c r="D9" s="46" t="n">
+        <v>14.57</v>
+      </c>
+      <c r="E9" s="46" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="F9" s="45" t="n">
+        <v>12.65</v>
+      </c>
+      <c r="G9" s="48" t="inlineStr">
+        <is>
+          <t>Equity Scheme - ELSS</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="28" t="inlineStr">
         <is>
-          <t>Gold BeES</t>
-        </is>
-      </c>
-      <c r="B10" s="29" t="n">
-        <v>115.49</v>
-      </c>
-      <c r="C10" s="35" t="n">
-        <v>57.07</v>
-      </c>
-      <c r="D10" s="35" t="n">
-        <v>143.6</v>
-      </c>
-      <c r="E10" s="35" t="n">
-        <v>196.97</v>
-      </c>
-      <c r="F10" s="35" t="inlineStr"/>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="28" t="inlineStr">
-        <is>
-          <t>Silver BeES</t>
-        </is>
-      </c>
-      <c r="B11" s="29" t="n">
-        <v>212.31</v>
-      </c>
-      <c r="C11" s="35" t="n">
-        <v>120.06</v>
-      </c>
-      <c r="D11" s="35" t="n">
-        <v>239.8</v>
-      </c>
-      <c r="E11" s="35" t="n">
-        <v>243.71</v>
-      </c>
-      <c r="F11" s="35" t="inlineStr"/>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="28" t="inlineStr">
-        <is>
-          <t>IT BeES</t>
-        </is>
-      </c>
-      <c r="B12" s="29" t="n">
-        <v>32.76</v>
-      </c>
-      <c r="C12" s="35" t="n">
-        <v>-16.98</v>
-      </c>
-      <c r="D12" s="35" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="E12" s="35" t="n">
-        <v>26.88</v>
-      </c>
-      <c r="F12" s="35" t="inlineStr"/>
+          <t xml:space="preserve">Taurus Flexi Cap Fund - Regular Plan - Growth </t>
+        </is>
+      </c>
+      <c r="B10" s="45" t="n">
+        <v>205.26</v>
+      </c>
+      <c r="C10" s="46" t="n">
+        <v>-3.98</v>
+      </c>
+      <c r="D10" s="46" t="n">
+        <v>13.73</v>
+      </c>
+      <c r="E10" s="46" t="n">
+        <v>10.92</v>
+      </c>
+      <c r="F10" s="46" t="n">
+        <v>9.609999999999999</v>
+      </c>
+      <c r="G10" s="48" t="inlineStr">
+        <is>
+          <t>Equity Scheme - Flexi Cap Fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="49" t="inlineStr">
+        <is>
+          <t>— ETFs &amp; BeES —</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="28" t="inlineStr">
         <is>
-          <t>Junior BeES</t>
+          <t>Nifty BeES</t>
         </is>
       </c>
       <c r="B13" s="29" t="n">
-        <v>672.29</v>
+        <v>259.83</v>
       </c>
       <c r="C13" s="35" t="n">
-        <v>5.78</v>
+        <v>3.03</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>70.43000000000001</v>
+        <v>36.97</v>
       </c>
       <c r="E13" s="35" t="n">
-        <v>91.26000000000001</v>
+        <v>68.87</v>
       </c>
       <c r="F13" s="35" t="inlineStr"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="28" t="inlineStr">
         <is>
-          <t>SBI Nifty ETF</t>
+          <t>Bank BeES</t>
         </is>
       </c>
       <c r="B14" s="29" t="n">
-        <v>245.18</v>
+        <v>543.04</v>
       </c>
       <c r="C14" s="35" t="n">
-        <v>2.96</v>
+        <v>9.51</v>
       </c>
       <c r="D14" s="35" t="n">
-        <v>36.66</v>
+        <v>33.08</v>
       </c>
       <c r="E14" s="35" t="n">
-        <v>68.17</v>
+        <v>63.06</v>
       </c>
       <c r="F14" s="35" t="inlineStr"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="28" t="inlineStr">
         <is>
-          <t>Momentum 100</t>
+          <t>Gold BeES</t>
         </is>
       </c>
       <c r="B15" s="29" t="n">
-        <v>58.39</v>
+        <v>115.49</v>
       </c>
       <c r="C15" s="35" t="n">
-        <v>12.2</v>
+        <v>57.07</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>83.67</v>
+        <v>143.6</v>
       </c>
       <c r="E15" s="35" t="n">
-        <v>136.78</v>
+        <v>196.97</v>
       </c>
       <c r="F15" s="35" t="inlineStr"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="28" t="inlineStr">
         <is>
-          <t>Hang Seng BeES</t>
+          <t>Silver BeES</t>
         </is>
       </c>
       <c r="B16" s="29" t="n">
-        <v>461.13</v>
+        <v>212.31</v>
       </c>
       <c r="C16" s="35" t="n">
-        <v>5.87</v>
+        <v>120.06</v>
       </c>
       <c r="D16" s="35" t="n">
-        <v>61.62</v>
+        <v>239.8</v>
       </c>
       <c r="E16" s="35" t="n">
-        <v>33.14</v>
+        <v>243.71</v>
       </c>
       <c r="F16" s="35" t="inlineStr"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="28" t="inlineStr">
         <is>
+          <t>IT BeES</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="n">
+        <v>32.76</v>
+      </c>
+      <c r="C17" s="35" t="n">
+        <v>-16.98</v>
+      </c>
+      <c r="D17" s="35" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E17" s="35" t="n">
+        <v>26.88</v>
+      </c>
+      <c r="F17" s="35" t="inlineStr"/>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>Junior BeES</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="n">
+        <v>672.29</v>
+      </c>
+      <c r="C18" s="35" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="D18" s="35" t="n">
+        <v>70.43000000000001</v>
+      </c>
+      <c r="E18" s="35" t="n">
+        <v>91.26000000000001</v>
+      </c>
+      <c r="F18" s="35" t="inlineStr"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>SBI Nifty ETF</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="n">
+        <v>245.18</v>
+      </c>
+      <c r="C19" s="35" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="D19" s="35" t="n">
+        <v>36.66</v>
+      </c>
+      <c r="E19" s="35" t="n">
+        <v>68.17</v>
+      </c>
+      <c r="F19" s="35" t="inlineStr"/>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>Momentum 100</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="C20" s="35" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="D20" s="35" t="n">
+        <v>83.67</v>
+      </c>
+      <c r="E20" s="35" t="n">
+        <v>136.78</v>
+      </c>
+      <c r="F20" s="35" t="inlineStr"/>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>Hang Seng BeES</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="n">
+        <v>461.13</v>
+      </c>
+      <c r="C21" s="35" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="D21" s="35" t="n">
+        <v>61.62</v>
+      </c>
+      <c r="E21" s="35" t="n">
+        <v>33.14</v>
+      </c>
+      <c r="F21" s="35" t="inlineStr"/>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
           <t>Bharat Bond 2032</t>
         </is>
       </c>
-      <c r="B17" s="29" t="n">
+      <c r="B22" s="29" t="n">
         <v>114.47</v>
       </c>
-      <c r="C17" s="35" t="n">
+      <c r="C22" s="35" t="n">
         <v>15.57</v>
       </c>
-      <c r="D17" s="35" t="n">
+      <c r="D22" s="35" t="n">
         <v>97.16</v>
       </c>
-      <c r="E17" s="35" t="n">
+      <c r="E22" s="35" t="n">
         <v>226.96</v>
       </c>
-      <c r="F17" s="35" t="inlineStr"/>
+      <c r="F22" s="35" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A12:G12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>